<commit_message>
Objective gradients are suppresed if constraints are violated.
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/LSR_20251119_all_materials.xlsx
+++ b/DataVaryingTemperature/LSR_20251119_all_materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deidum\METALS\Results\20251118_delivery_to_WI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0FE14E0-57D4-4C12-BB5D-00EF0F72F1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E927CEA-6288-47CD-BB79-9833F4DCF5B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t>Attribute</t>
   </si>
@@ -181,15 +181,6 @@
   </si>
   <si>
     <t>Fatigue_Limit</t>
-  </si>
-  <si>
-    <t>Granta Selector</t>
-  </si>
-  <si>
-    <t>Inverse Analysis</t>
-  </si>
-  <si>
-    <t>Calculated</t>
   </si>
 </sst>
 </file>
@@ -613,24 +604,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:V18"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="9.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="1" customWidth="1"/>
-    <col min="8" max="10" width="11.7109375" style="1" customWidth="1"/>
-    <col min="11" max="14" width="10.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8" max="10" width="11.6640625" style="1" customWidth="1"/>
+    <col min="11" max="14" width="10.44140625" style="1" customWidth="1"/>
     <col min="15" max="15" width="10" style="1" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="16.5703125" style="1" customWidth="1"/>
-    <col min="18" max="705" width="20.5703125" style="1" customWidth="1"/>
-    <col min="706" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="16" width="13.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="16.5546875" style="1" customWidth="1"/>
+    <col min="18" max="704" width="20.5546875" style="1" customWidth="1"/>
+    <col min="705" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
       <c r="B1" s="6" t="s">
         <v>4</v>
@@ -684,7 +675,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="7" t="s">
         <v>7</v>
@@ -738,7 +729,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>34</v>
       </c>
@@ -751,23 +742,27 @@
       <c r="D3" s="17">
         <v>31660210473.422401</v>
       </c>
-      <c r="E3" s="17">
-        <v>73276522231.125107</v>
-      </c>
-      <c r="F3" s="17">
-        <v>42098834999.111099</v>
-      </c>
-      <c r="G3" s="17">
+      <c r="E3" s="12">
+        <f>D3*EXP(-2000/Q3)</f>
+        <v>318975670.52076489</v>
+      </c>
+      <c r="F3" s="12">
+        <f>0.1*D3*EXP(-3000/Q3)</f>
+        <v>3201691.1808246872</v>
+      </c>
+      <c r="G3" s="12">
         <v>1.0001904096107801</v>
       </c>
-      <c r="H3" s="17">
+      <c r="H3" s="12">
         <v>168216570.304768</v>
       </c>
-      <c r="I3" s="17">
-        <v>1626009334.9888</v>
-      </c>
-      <c r="J3" s="17">
-        <v>1362827.91216376</v>
+      <c r="I3" s="12">
+        <f>0.1*H3*EXP(-2000/Q3)</f>
+        <v>169477.68982998349</v>
+      </c>
+      <c r="J3" s="12">
+        <f>0.1*H3*EXP(-3000/Q3)</f>
+        <v>17011.179065454031</v>
       </c>
       <c r="K3" s="17">
         <v>1.0002813979562399</v>
@@ -787,14 +782,14 @@
       <c r="P3" s="15">
         <v>0.25</v>
       </c>
-      <c r="Q3" s="7">
-        <v>150</v>
+      <c r="Q3" s="12">
+        <v>435</v>
       </c>
       <c r="R3" s="8">
         <v>112000000</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -808,10 +803,12 @@
         <v>88122361302.941193</v>
       </c>
       <c r="E4" s="12">
-        <v>43160916887.095703</v>
+        <f t="shared" ref="E4:E5" si="0">D4*EXP(-2000/Q4)</f>
+        <v>425450353.708947</v>
       </c>
       <c r="F4" s="12">
-        <v>2048198742574.49</v>
+        <f t="shared" ref="F4:F5" si="1">0.1*D4*EXP(-3000/Q4)</f>
+        <v>2956175.8899659268</v>
       </c>
       <c r="G4" s="12">
         <v>0.99968676964325098</v>
@@ -820,10 +817,12 @@
         <v>331895501.95574099</v>
       </c>
       <c r="I4" s="12">
-        <v>411398268.51887101</v>
+        <f t="shared" ref="I4:I5" si="2">0.1*H4*EXP(-2000/Q4)</f>
+        <v>160237.4886619903</v>
       </c>
       <c r="J4" s="12">
-        <v>211126489.35119501</v>
+        <f t="shared" ref="J4:J5" si="3">0.1*H4*EXP(-3000/Q4)</f>
+        <v>11133.853727509615</v>
       </c>
       <c r="K4" s="12">
         <v>1.00011111067342</v>
@@ -843,14 +842,14 @@
       <c r="P4" s="15">
         <v>0.74</v>
       </c>
-      <c r="Q4" s="7">
-        <v>150</v>
+      <c r="Q4" s="12">
+        <v>375</v>
       </c>
       <c r="R4" s="8">
         <v>118000000</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>36</v>
       </c>
@@ -864,10 +863,12 @@
         <v>92976880986.810806</v>
       </c>
       <c r="E5" s="12">
-        <v>36504792717.403801</v>
+        <f t="shared" si="0"/>
+        <v>306684777.10425931</v>
       </c>
       <c r="F5" s="12">
-        <v>2472842900671.1802</v>
+        <f t="shared" si="1"/>
+        <v>1761371.0038603023</v>
       </c>
       <c r="G5" s="12">
         <v>0.99992423656867901</v>
@@ -876,10 +877,12 @@
         <v>413532439.30818099</v>
       </c>
       <c r="I5" s="12">
-        <v>478670621.39346302</v>
+        <f t="shared" si="2"/>
+        <v>136403.9131325568</v>
       </c>
       <c r="J5" s="12">
-        <v>10759114.630594</v>
+        <f t="shared" si="3"/>
+        <v>7834.0340095552874</v>
       </c>
       <c r="K5" s="12">
         <v>1.0004243155682</v>
@@ -899,14 +902,14 @@
       <c r="P5" s="15">
         <v>0.15</v>
       </c>
-      <c r="Q5" s="7">
-        <v>200</v>
+      <c r="Q5" s="12">
+        <v>350</v>
       </c>
       <c r="R5" s="8">
         <v>150000000</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>37</v>
       </c>
@@ -955,16 +958,16 @@
       <c r="P6" s="15">
         <v>0.46</v>
       </c>
-      <c r="Q6" s="7">
-        <v>400</v>
+      <c r="Q6" s="12">
+        <v>1050</v>
       </c>
       <c r="R6" s="8">
         <v>229000000</v>
       </c>
-      <c r="U6" s="5"/>
-      <c r="W6" s="5"/>
-    </row>
-    <row r="7" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="T6" s="5"/>
+      <c r="V6" s="5"/>
+    </row>
+    <row r="7" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>38</v>
       </c>
@@ -1013,14 +1016,14 @@
       <c r="P7" s="15">
         <v>0.41</v>
       </c>
-      <c r="Q7" s="7">
-        <v>399</v>
+      <c r="Q7" s="12">
+        <v>1050</v>
       </c>
       <c r="R7" s="8">
         <v>229000000</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
@@ -1069,14 +1072,14 @@
       <c r="P8" s="15">
         <v>0.36</v>
       </c>
-      <c r="Q8" s="7">
-        <v>316</v>
+      <c r="Q8" s="12">
+        <v>1050</v>
       </c>
       <c r="R8" s="8">
         <v>364000000</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>40</v>
       </c>
@@ -1125,14 +1128,14 @@
       <c r="P9" s="15">
         <v>0.35</v>
       </c>
-      <c r="Q9" s="7">
-        <v>632</v>
+      <c r="Q9" s="12">
+        <v>1040</v>
       </c>
       <c r="R9" s="8">
         <v>407000000</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>41</v>
       </c>
@@ -1181,14 +1184,14 @@
       <c r="P10" s="15">
         <v>0.64</v>
       </c>
-      <c r="Q10" s="7">
-        <v>700</v>
+      <c r="Q10" s="12">
+        <v>1000</v>
       </c>
       <c r="R10" s="8">
         <v>485000000</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>42</v>
       </c>
@@ -1237,14 +1240,14 @@
       <c r="P11" s="15">
         <v>1E-3</v>
       </c>
-      <c r="Q11" s="7">
-        <v>330</v>
+      <c r="Q11" s="12">
+        <v>1200</v>
       </c>
       <c r="R11" s="8">
         <v>245000000</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>43</v>
       </c>
@@ -1293,27 +1296,21 @@
       <c r="P12" s="15">
         <v>1E-3</v>
       </c>
-      <c r="Q12" s="7">
-        <v>330</v>
+      <c r="Q12" s="12">
+        <v>1200</v>
       </c>
       <c r="R12" s="8">
         <v>245000000</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B16" s="13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="16" t="s">
-        <v>48</v>
-      </c>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="B16" s="13"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="9"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1334,12 +1331,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC80EBF-8B96-4896-8C13-AD8A976D05A3}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1353,7 +1350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1367,7 +1364,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1381,7 +1378,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1395,7 +1392,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>

</xml_diff>